<commit_message>
first llm journal tier rankings included
</commit_message>
<xml_diff>
--- a/data/UJ_map.xlsx
+++ b/data/UJ_map.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2333" uniqueCount="1067">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2332" uniqueCount="1068">
   <si>
     <t>Acemoglu et al. 2024</t>
   </si>
@@ -3251,6 +3251,9 @@
   </si>
   <si>
     <t>A Welfare Analysis of Policies Impacting Climate Change</t>
+  </si>
+  <si>
+    <t>Blimpo and Castaneda-Dower 2025</t>
   </si>
 </sst>
 </file>
@@ -4028,27 +4031,26 @@
       </c>
     </row>
     <row r="50" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="8" t="s">
+        <v>1067</v>
+      </c>
       <c r="B50" s="8" t="s">
         <v>1065</v>
       </c>
     </row>
     <row r="51" spans="1:3" s="8" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B51" s="7" t="s">
-        <v>1066</v>
-      </c>
       <c r="C51" s="7"/>
     </row>
-    <row r="52" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="8" t="s">
-        <v>1066</v>
-      </c>
-    </row>
+    <row r="52" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="53" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="54" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="55" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="56" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="57" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="58" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A58"/>
+      <c r="B58"/>
+    </row>
   </sheetData>
   <sortState ref="A2:B47">
     <sortCondition ref="B2:B47"/>

</xml_diff>